<commit_message>
feat: add Micro-Market sheet + missing costs to Startup Costs
- New "Micro-Market Costs" sheet: honesty shop / unsupervised retail
  scenario with fridge, shelving, payment terminal, shrinkage budget,
  waste/spoilage line, and side-by-side comparison vs vending
- Startup Costs: added customer acquisition costs, accountant, SIM/data,
  printed materials, updated Nayax to confirmed £450
- Dashboard references updated to correct rows
- All cross-sheet formulas verified

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TheSnackChoice_London_Research.xlsx
+++ b/TheSnackChoice_London_Research.xlsx
@@ -13,8 +13,9 @@
     <sheet name="Supplier Directory" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Competitor Analysis" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Startup Costs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Location Tracker" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Weekly P&amp;L" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Micro-Market Costs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Location Tracker" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Weekly P&amp;L" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Product Catalog'!$A$1:$N$60</definedName>
@@ -80,7 +81,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +106,12 @@
         <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,6 +159,10 @@
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -609,7 +620,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>'Startup Costs'!D35</f>
+        <f>'Startup Costs'!D39</f>
         <v/>
       </c>
     </row>
@@ -620,7 +631,7 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>'Startup Costs'!D32</f>
+        <f>'Startup Costs'!D36</f>
         <v/>
       </c>
     </row>
@@ -631,7 +642,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>'Startup Costs'!D38</f>
+        <f>'Startup Costs'!D42</f>
         <v/>
       </c>
     </row>
@@ -642,7 +653,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>'Startup Costs'!D39</f>
+        <f>'Startup Costs'!D43</f>
         <v/>
       </c>
     </row>
@@ -653,7 +664,7 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>'Startup Costs'!D40</f>
+        <f>'Startup Costs'!D44</f>
         <v/>
       </c>
     </row>
@@ -7842,7 +7853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8123,7 +8134,7 @@
       </c>
       <c r="E17" s="24" t="inlineStr">
         <is>
-          <t>£1-2M cover</t>
+          <t>£1-2M cover — get quotes, may be £300-600</t>
         </is>
       </c>
     </row>
@@ -8218,70 +8229,87 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Printed Materials (leaflets/cards)</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="C22" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="7">
+        <f>B22*C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>For site pitching</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Customer Acquisition (time/fuel)</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="C23" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D23" s="7">
+        <f>B23*C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>£100 per placed machine — ~10 pitches per win</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Subtotal Setup</t>
         </is>
       </c>
-      <c r="D22" s="23">
-        <f>SUM(D14:D21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="D24" s="23">
+        <f>SUM(D14:D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>MONTHLY OPERATING COSTS</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>Per Machine/Month (£)</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>Total/Month (£)</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="21" t="inlineStr">
-        <is>
-          <t>Nayax Monthly Fee</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D25" s="7">
-        <f>B25*$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>Site Rent / Commission</t>
-        </is>
-      </c>
-      <c r="B26" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="D26" s="7">
-        <f>B26*$B$2</f>
-        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="21" t="inlineStr">
         <is>
-          <t>Stock Replenishment</t>
-        </is>
-      </c>
-      <c r="B27" s="22" t="n">
-        <v>400</v>
+          <t>Nayax Monthly Fee</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>10</v>
       </c>
       <c r="D27" s="7">
         <f>B27*$B$2</f>
@@ -8291,11 +8319,11 @@
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>Travel/Fuel</t>
-        </is>
-      </c>
-      <c r="B28" s="22" t="n">
-        <v>80</v>
+          <t>Nayax SIM/Data</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="D28" s="7">
         <f>B28*$B$2</f>
@@ -8305,11 +8333,11 @@
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>Electricity (if not site-covered)</t>
+          <t>Site Rent / Commission</t>
         </is>
       </c>
       <c r="B29" s="22" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D29" s="7">
         <f>B29*$B$2</f>
@@ -8319,11 +8347,11 @@
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
         <is>
-          <t>Maintenance/Repairs Fund</t>
+          <t>Stock Replenishment</t>
         </is>
       </c>
       <c r="B30" s="22" t="n">
-        <v>30</v>
+        <v>400</v>
       </c>
       <c r="D30" s="7">
         <f>B30*$B$2</f>
@@ -8333,104 +8361,160 @@
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
+          <t>Travel/Fuel</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="n">
+        <v>80</v>
+      </c>
+      <c r="D31" s="7">
+        <f>B31*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Electricity (if not site-covered)</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="7">
+        <f>B32*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Maintenance/Repairs Fund</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="D33" s="7">
+        <f>B33*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Accountant (pro-rata monthly)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D34" s="7">
+        <f>B34*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
           <t>Misc/Phone/Admin</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B35" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="D31" s="7">
-        <f>B31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Total Monthly Opex</t>
-        </is>
-      </c>
-      <c r="D32" s="23">
-        <f>SUM(D25:D31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>SUMMARY</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Total Upfront Investment</t>
-        </is>
-      </c>
-      <c r="D35" s="23">
-        <f>D11+D22</f>
+      <c r="D35" s="7">
+        <f>B35</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Monthly Operating Cost</t>
+          <t>Total Monthly Opex</t>
         </is>
       </c>
       <c r="D36" s="23">
-        <f>D32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Est. Monthly Revenue per Machine</t>
-        </is>
-      </c>
-      <c r="B37" s="22" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D37" s="23">
-        <f>B37*$B$2</f>
+        <f>SUM(D27:D35)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Est. Monthly Revenue Total</t>
-        </is>
-      </c>
-      <c r="D38" s="23">
-        <f>D37</f>
-        <v/>
-      </c>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Est. Monthly Profit</t>
+          <t>Total Upfront Investment</t>
         </is>
       </c>
       <c r="D39" s="23">
-        <f>D38-D36</f>
+        <f>D11+D24</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
+          <t>Monthly Operating Cost</t>
+        </is>
+      </c>
+      <c r="D40" s="23">
+        <f>D36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Est. Monthly Revenue per Machine</t>
+        </is>
+      </c>
+      <c r="B41" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D41" s="23">
+        <f>B41*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Est. Monthly Revenue Total</t>
+        </is>
+      </c>
+      <c r="D42" s="23">
+        <f>D41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Est. Monthly Profit</t>
+        </is>
+      </c>
+      <c r="D43" s="23">
+        <f>D42-D40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
           <t>Months to Breakeven</t>
         </is>
       </c>
-      <c r="D40" s="8">
-        <f>D35/D39</f>
+      <c r="D44" s="8">
+        <f>D39/D43</f>
         <v/>
       </c>
     </row>
@@ -8440,6 +8524,712 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>MICRO-MARKET / HONESTY SHOP CALCULATOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Number of sites:</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CAPITAL COSTS (PER SITE)</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Per Site (£)</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Total (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Commercial Fridge (undercounter/upright)</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="n">
+        <v>350</v>
+      </c>
+      <c r="C5" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D5" s="7">
+        <f>B5*C5</f>
+        <v/>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Argos/Amazon Business</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Shelving Unit</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D6" s="7">
+        <f>B6*C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Freestanding or wall-mounted</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Payment Terminal (scanner/card reader)</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="n">
+        <v>400</v>
+      </c>
+      <c r="C7" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D7" s="7">
+        <f>B7*C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>SumUp Kiosk / Nayax / PayPoint — TBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>VAT on Equipment</t>
+        </is>
+      </c>
+      <c r="B8" s="7">
+        <f>SUM(B5:B7)*0.2</f>
+        <v/>
+      </c>
+      <c r="C8" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>B8*C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>20% on above</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Signage &amp; Branding</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D9" s="7">
+        <f>B9*C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>Price labels, branding board</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Initial Stock Fill</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="n">
+        <v>250</v>
+      </c>
+      <c r="C10" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D10" s="7">
+        <f>B10*C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>Wider range than vending</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Subtotal Capital</t>
+        </is>
+      </c>
+      <c r="D11" s="23">
+        <f>SUM(D5:D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>SETUP COSTS (ONE-OFF)</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>Cost (£)</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Total (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Company Registration (Ltd)</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7">
+        <f>B14*C14</f>
+        <v/>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Shared with vending if same entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Food Business Registration</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="7">
+        <f>B15*C15</f>
+        <v/>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Free, local council</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Food Hygiene Certificate</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="n">
+        <v>150</v>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="7">
+        <f>B16*C16</f>
+        <v/>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>Level 2 online course</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Public Liability Insurance (annual)</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7">
+        <f>B17*C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>May be higher for open shelving</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Product Liability Insurance (annual)</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7">
+        <f>B18*C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>Covers consumed products</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>Printed Materials</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7">
+        <f>B19*C19</f>
+        <v/>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>Leaflets for site pitching</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Customer Acquisition (time/fuel)</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="C20" s="21">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D20" s="7">
+        <f>B20*C20</f>
+        <v/>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>Per site placed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Subtotal Setup</t>
+        </is>
+      </c>
+      <c r="D21" s="23">
+        <f>SUM(D14:D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>MONTHLY OPERATING COSTS</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>Per Site/Month (£)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>Total/Month (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Payment Terminal Fee</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" s="7">
+        <f>B24*$B$2</f>
+        <v/>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>Monthly subscription</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Site Rent / Commission</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="D25" s="7">
+        <f>B25*$B$2</f>
+        <v/>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Often lower than vending — you supply product</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Stock Replenishment</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="n">
+        <v>500</v>
+      </c>
+      <c r="D26" s="7">
+        <f>B26*$B$2</f>
+        <v/>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>Higher volume, wider range</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>Shrinkage Budget (3-5%)</t>
+        </is>
+      </c>
+      <c r="B27" s="7">
+        <f>B26*0.04</f>
+        <v/>
+      </c>
+      <c r="D27" s="7">
+        <f>B27*$B$2</f>
+        <v/>
+      </c>
+      <c r="E27" s="24">
+        <f>stock * shrinkage rate</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Travel/Fuel</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="n">
+        <v>60</v>
+      </c>
+      <c r="D28" s="7">
+        <f>B28*$B$2</f>
+        <v/>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>Faster restock = fewer visits</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>Waste/Spoilage (fresh food)</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="D29" s="7">
+        <f>B29*$B$2</f>
+        <v/>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Set to 0 if no fresh items</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Accountant (pro-rata monthly)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D30" s="7">
+        <f>B30</f>
+        <v/>
+      </c>
+      <c r="E30" s="24" t="inlineStr">
+        <is>
+          <t>Shared with vending if same entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>Misc/Phone/Admin</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D31" s="7">
+        <f>B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Total Monthly Opex</t>
+        </is>
+      </c>
+      <c r="D32" s="23">
+        <f>SUM(D24:D31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Total Upfront Investment</t>
+        </is>
+      </c>
+      <c r="D35" s="23">
+        <f>D11+D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Monthly Operating Cost</t>
+        </is>
+      </c>
+      <c r="D36" s="23">
+        <f>D32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Est. Monthly Revenue per Site</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D37" s="23">
+        <f>B37*$B$2</f>
+        <v/>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>Higher avg basket than vending</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Est. Monthly Revenue Total</t>
+        </is>
+      </c>
+      <c r="D38" s="23">
+        <f>D37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Est. Monthly Profit</t>
+        </is>
+      </c>
+      <c r="D39" s="23">
+        <f>D38-D36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Months to Breakeven</t>
+        </is>
+      </c>
+      <c r="D40" s="25">
+        <f>D35/D39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>VS VENDING (from Startup Costs sheet)</t>
+        </is>
+      </c>
+      <c r="B42" s="27" t="n"/>
+      <c r="C42" s="27" t="n"/>
+      <c r="D42" s="27" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Vending: Upfront Investment</t>
+        </is>
+      </c>
+      <c r="D43" s="10">
+        <f>'Startup Costs'!D39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Micro-Market: Upfront Investment</t>
+        </is>
+      </c>
+      <c r="D44" s="10">
+        <f>D35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="inlineStr">
+        <is>
+          <t>Capital Saving</t>
+        </is>
+      </c>
+      <c r="D45" s="28">
+        <f>D43-D44</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8620,7 +9410,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8661,7 +9451,7 @@
           <t>Week Commencing:</t>
         </is>
       </c>
-      <c r="B3" s="25" t="n"/>
+      <c r="B3" s="29" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -8711,8 +9501,8 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="B6" s="26" t="n"/>
-      <c r="C6" s="26" t="n"/>
+      <c r="B6" s="30" t="n"/>
+      <c r="C6" s="30" t="n"/>
       <c r="D6" s="14">
         <f>B6+C6</f>
         <v/>
@@ -8734,8 +9524,8 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n"/>
-      <c r="C7" s="26" t="n"/>
+      <c r="B7" s="30" t="n"/>
+      <c r="C7" s="30" t="n"/>
       <c r="D7" s="14">
         <f>B7+C7</f>
         <v/>
@@ -8757,8 +9547,8 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="26" t="n"/>
+      <c r="B8" s="30" t="n"/>
+      <c r="C8" s="30" t="n"/>
       <c r="D8" s="14">
         <f>B8+C8</f>
         <v/>
@@ -8780,8 +9570,8 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n"/>
-      <c r="C9" s="26" t="n"/>
+      <c r="B9" s="30" t="n"/>
+      <c r="C9" s="30" t="n"/>
       <c r="D9" s="14">
         <f>B9+C9</f>
         <v/>
@@ -8803,8 +9593,8 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
+      <c r="B10" s="30" t="n"/>
+      <c r="C10" s="30" t="n"/>
       <c r="D10" s="14">
         <f>B10+C10</f>
         <v/>
@@ -8826,8 +9616,8 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n"/>
-      <c r="C11" s="26" t="n"/>
+      <c r="B11" s="30" t="n"/>
+      <c r="C11" s="30" t="n"/>
       <c r="D11" s="14">
         <f>B11+C11</f>
         <v/>
@@ -8849,8 +9639,8 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B12" s="26" t="n"/>
-      <c r="C12" s="26" t="n"/>
+      <c r="B12" s="30" t="n"/>
+      <c r="C12" s="30" t="n"/>
       <c r="D12" s="14">
         <f>B12+C12</f>
         <v/>
@@ -8872,15 +9662,15 @@
           <t>WEEK TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="31">
         <f>SUM(B6:B12)</f>
         <v/>
       </c>
-      <c r="C13" s="27">
+      <c r="C13" s="31">
         <f>SUM(C6:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="31">
         <f>SUM(D6:D12)</f>
         <v/>
       </c>
@@ -8896,7 +9686,7 @@
         <f>SUM(G6:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="31">
         <f>IF(G13=0,"",D13/G13)</f>
         <v/>
       </c>
@@ -8919,7 +9709,7 @@
           <t>Stock Purchased</t>
         </is>
       </c>
-      <c r="B16" s="28" t="n"/>
+      <c r="B16" s="32" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="21" t="inlineStr">
@@ -8927,7 +9717,7 @@
           <t>Card Processing Fees</t>
         </is>
       </c>
-      <c r="B17" s="29">
+      <c r="B17" s="33">
         <f>SUM(C6:C12)*0.029</f>
         <v/>
       </c>
@@ -8938,7 +9728,7 @@
           <t>Nayax Monthly (pro-rata weekly)</t>
         </is>
       </c>
-      <c r="B18" s="29">
+      <c r="B18" s="33">
         <f>10/4.33</f>
         <v/>
       </c>
@@ -8949,7 +9739,7 @@
           <t>Site Rent (pro-rata weekly)</t>
         </is>
       </c>
-      <c r="B19" s="28" t="n"/>
+      <c r="B19" s="32" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="21" t="inlineStr">
@@ -8957,7 +9747,7 @@
           <t>Travel/Fuel</t>
         </is>
       </c>
-      <c r="B20" s="28" t="n"/>
+      <c r="B20" s="32" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="21" t="inlineStr">
@@ -8965,7 +9755,7 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="B21" s="28" t="n"/>
+      <c r="B21" s="32" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -8973,7 +9763,7 @@
           <t>Total Costs</t>
         </is>
       </c>
-      <c r="B22" s="30">
+      <c r="B22" s="34">
         <f>SUM(B16:B21)</f>
         <v/>
       </c>
@@ -8992,7 +9782,7 @@
           <t>Gross Revenue</t>
         </is>
       </c>
-      <c r="B25" s="27">
+      <c r="B25" s="31">
         <f>D13</f>
         <v/>
       </c>
@@ -9003,7 +9793,7 @@
           <t>Total Costs</t>
         </is>
       </c>
-      <c r="B26" s="27">
+      <c r="B26" s="31">
         <f>B22</f>
         <v/>
       </c>
@@ -9014,7 +9804,7 @@
           <t>Net Profit</t>
         </is>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="31">
         <f>B25-B26</f>
         <v/>
       </c>
@@ -9025,7 +9815,7 @@
           <t>Gross Margin %</t>
         </is>
       </c>
-      <c r="B28" s="31">
+      <c r="B28" s="35">
         <f>IF(B25=0,"",(B25-B16)/B25)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat: add Operations Log + Performance Review sheets
Behold loop applied to vending operations:

- Operations Log: restock/visit log, maintenance log, operational
  beliefs (WHY — review quarterly), operational methods (HOW —
  review monthly with editable settings)
- Performance Review: site performance (weekly rev/hour tracking),
  product performance (monthly with keep/replace/drop actions),
  monthly review gate (Observe → Orient → Decide → Act → Protect)
  with the key rule: one change at a time, wait 4 weeks, measure

Conditional formatting on revenue-per-hour (red <£15, green >£30)
to surface underperforming sites immediately.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TheSnackChoice_London_Research.xlsx
+++ b/TheSnackChoice_London_Research.xlsx
@@ -16,6 +16,8 @@
     <sheet name="Micro-Market Costs" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Location Tracker" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Weekly P&amp;L" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Operations Log" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Performance Review" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Product Catalog'!$A$1:$N$60</definedName>
@@ -33,7 +35,7 @@
     <numFmt numFmtId="167" formatCode="£#,##0.00"/>
     <numFmt numFmtId="168" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +81,16 @@
       <i val="1"/>
       <color rgb="00808080"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -131,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -170,6 +182,12 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -918,6 +936,1409 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>RESTOCK &amp; VISIT LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Machine/Site ID</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Visit Type</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Time Spent (min)</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Mileage</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Items Restocked (summary)</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Issues Found</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Cost of Stock (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="36" t="n"/>
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="37" t="n"/>
+      <c r="F3" s="38" t="n"/>
+      <c r="G3" s="16" t="n"/>
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="13" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="36" t="n"/>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="37" t="n"/>
+      <c r="F4" s="38" t="n"/>
+      <c r="G4" s="16" t="n"/>
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="13" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="36" t="n"/>
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="37" t="n"/>
+      <c r="F5" s="38" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="13" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="n"/>
+      <c r="B6" s="16" t="n"/>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="37" t="n"/>
+      <c r="F6" s="38" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="13" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="36" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="37" t="n"/>
+      <c r="F7" s="38" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="13" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="n"/>
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="16" t="n"/>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="37" t="n"/>
+      <c r="F8" s="38" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="16" t="n"/>
+      <c r="I8" s="13" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="36" t="n"/>
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="37" t="n"/>
+      <c r="F9" s="38" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="16" t="n"/>
+      <c r="I9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="n"/>
+      <c r="B10" s="16" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="37" t="n"/>
+      <c r="F10" s="38" t="n"/>
+      <c r="G10" s="16" t="n"/>
+      <c r="H10" s="16" t="n"/>
+      <c r="I10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="36" t="n"/>
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="37" t="n"/>
+      <c r="F11" s="38" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="16" t="n"/>
+      <c r="I11" s="13" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="36" t="n"/>
+      <c r="B12" s="16" t="n"/>
+      <c r="C12" s="16" t="n"/>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="37" t="n"/>
+      <c r="F12" s="38" t="n"/>
+      <c r="G12" s="16" t="n"/>
+      <c r="H12" s="16" t="n"/>
+      <c r="I12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="36" t="n"/>
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="16" t="n"/>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="37" t="n"/>
+      <c r="F13" s="38" t="n"/>
+      <c r="G13" s="16" t="n"/>
+      <c r="H13" s="16" t="n"/>
+      <c r="I13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="n"/>
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="37" t="n"/>
+      <c r="F14" s="38" t="n"/>
+      <c r="G14" s="16" t="n"/>
+      <c r="H14" s="16" t="n"/>
+      <c r="I14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="36" t="n"/>
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="37" t="n"/>
+      <c r="F15" s="38" t="n"/>
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="16" t="n"/>
+      <c r="I15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="36" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="37" t="n"/>
+      <c r="F16" s="38" t="n"/>
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="16" t="n"/>
+      <c r="I16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="36" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="37" t="n"/>
+      <c r="F17" s="38" t="n"/>
+      <c r="G17" s="16" t="n"/>
+      <c r="H17" s="16" t="n"/>
+      <c r="I17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="36" t="n"/>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="37" t="n"/>
+      <c r="F18" s="38" t="n"/>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="16" t="n"/>
+      <c r="I18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="36" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="37" t="n"/>
+      <c r="F19" s="38" t="n"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>MAINTENANCE LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Machine/Site ID</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Fault Description</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Action Taken</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Parts Cost (£)</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Labour Cost (£)</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>Under Warranty</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36" t="n"/>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="16" t="n"/>
+      <c r="I24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="36" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="16" t="n"/>
+      <c r="I25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="16" t="n"/>
+      <c r="I26" s="16" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="36" t="n"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="16" t="n"/>
+      <c r="I27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="36" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="16" t="n"/>
+      <c r="I28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="36" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="16" t="n"/>
+      <c r="I29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="n"/>
+      <c r="B30" s="16" t="n"/>
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="16" t="n"/>
+      <c r="E30" s="16" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="16" t="n"/>
+      <c r="I30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="36" t="n"/>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="16" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="13" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="36" t="n"/>
+      <c r="B32" s="16" t="n"/>
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="16" t="n"/>
+      <c r="I32" s="16" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="36" t="n"/>
+      <c r="B33" s="16" t="n"/>
+      <c r="C33" s="16" t="n"/>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="13" t="n"/>
+      <c r="H33" s="16" t="n"/>
+      <c r="I33" s="16" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>OPERATIONAL BELIEFS (review quarterly)</t>
+        </is>
+      </c>
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="27" t="n"/>
+      <c r="D36" s="27" t="n"/>
+      <c r="E36" s="27" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>Cluster density over scattered reach</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>Add sites near existing ones. Revenue per hour of drive time is the real metric.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>Stock-out costs more than overstock</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>Empty slot = lost sale + trained-away customer. Overstocked shelf = zero cost (non-perishable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>Data-driven restocking, not calendar-driven</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Check Nayax/sales data before every run. Let demand set visit frequency, not habit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>Revenue per operator-hour is the north star</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>Track time spent per site. If a site takes 2 hours for £30/week revenue, drop it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>Every visit is a gate: observe, orient, act, log</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>Pre-visit: check dashboard. On-site: restock + inspect + clean. Post-visit: log anomalies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>OPERATIONAL METHODS (review monthly)</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="n"/>
+      <c r="C43" s="27" t="n"/>
+      <c r="D43" s="27" t="n"/>
+      <c r="E43" s="27" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>Current Setting</t>
+        </is>
+      </c>
+      <c r="C44" s="18" t="inlineStr">
+        <is>
+          <t>Last Reviewed</t>
+        </is>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Purchasing strategy</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="inlineStr">
+        <is>
+          <t>JIT (buy morning of restock)</t>
+        </is>
+      </c>
+      <c r="C45" s="39" t="inlineStr"/>
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>Switch to bulk when 5+ machines</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Restock frequency</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="inlineStr">
+        <is>
+          <t>2x/week per machine</t>
+        </is>
+      </c>
+      <c r="C46" s="39" t="inlineStr"/>
+      <c r="D46" s="24" t="inlineStr">
+        <is>
+          <t>Adjust per site based on Nayax data</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Product rotation cadence</t>
+        </is>
+      </c>
+      <c r="B47" s="19" t="inlineStr">
+        <is>
+          <t>Monthly — swap bottom 3 sellers</t>
+        </is>
+      </c>
+      <c r="C47" s="39" t="inlineStr"/>
+      <c r="D47" s="24" t="inlineStr">
+        <is>
+          <t>Track via Weekly P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Pricing strategy</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="inlineStr">
+        <is>
+          <t>60%+ net margin target</t>
+        </is>
+      </c>
+      <c r="C48" s="39" t="inlineStr"/>
+      <c r="D48" s="24" t="inlineStr">
+        <is>
+          <t>Premium sites can go higher</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Margin floor</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="inlineStr">
+        <is>
+          <t>30% net minimum to stock</t>
+        </is>
+      </c>
+      <c r="C49" s="39" t="inlineStr"/>
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t>Below this, product isn't worth the slot</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Visit time target</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="inlineStr">
+        <is>
+          <t>30 min per machine</t>
+        </is>
+      </c>
+      <c r="C50" s="39" t="inlineStr"/>
+      <c r="D50" s="24" t="inlineStr">
+        <is>
+          <t>Including travel, restock, clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Shrinkage threshold (micro-market)</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="inlineStr">
+        <is>
+          <t>5% — investigate above this</t>
+        </is>
+      </c>
+      <c r="C51" s="39" t="inlineStr"/>
+      <c r="D51" s="24" t="inlineStr">
+        <is>
+          <t>Camera or format change if persistent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="D3:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list" type="list">
+      <formula1>"Restock,Top-up,Maintenance,Inspection,Install,Removal,Emergency"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D24:D74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list" type="list">
+      <formula1>"Low,Medium,High,Critical"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H24:H74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list" type="list">
+      <formula1>"Yes,No,Pending Parts"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I24:I74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list" type="list">
+      <formula1>"Yes,No,Claim Submitted"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>PERFORMANCE REVIEW — THE ORIENTATION LOOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>Fill weekly. Review monthly. Beliefs and methods evolve from what you see here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SITE PERFORMANCE (weekly)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Machine/Site ID</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Week Commencing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Revenue (£)</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Stock Cost (£)</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Gross Margin (%)</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Vends/Day (est.)</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Operator Hours</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Revenue per Hour (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="n"/>
+      <c r="B6" s="36" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="9">
+        <f>IF(C6="","",(C6-D6)/C6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="38" t="n"/>
+      <c r="G6" s="38" t="n"/>
+      <c r="H6" s="14">
+        <f>IF(G6="","",C6/G6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n"/>
+      <c r="B7" s="36" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="9">
+        <f>IF(C7="","",(C7-D7)/C7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="38" t="n"/>
+      <c r="G7" s="38" t="n"/>
+      <c r="H7" s="14">
+        <f>IF(G7="","",C7/G7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="n"/>
+      <c r="B8" s="36" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="9">
+        <f>IF(C8="","",(C8-D8)/C8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="38" t="n"/>
+      <c r="G8" s="38" t="n"/>
+      <c r="H8" s="14">
+        <f>IF(G8="","",C8/G8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="n"/>
+      <c r="B9" s="36" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="9">
+        <f>IF(C9="","",(C9-D9)/C9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="38" t="n"/>
+      <c r="G9" s="38" t="n"/>
+      <c r="H9" s="14">
+        <f>IF(G9="","",C9/G9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="n"/>
+      <c r="B10" s="36" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="9">
+        <f>IF(C10="","",(C10-D10)/C10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="38" t="n"/>
+      <c r="G10" s="38" t="n"/>
+      <c r="H10" s="14">
+        <f>IF(G10="","",C10/G10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="n"/>
+      <c r="B11" s="36" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="9">
+        <f>IF(C11="","",(C11-D11)/C11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="38" t="n"/>
+      <c r="G11" s="38" t="n"/>
+      <c r="H11" s="14">
+        <f>IF(G11="","",C11/G11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n"/>
+      <c r="B12" s="36" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="9">
+        <f>IF(C12="","",(C12-D12)/C12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="38" t="n"/>
+      <c r="G12" s="38" t="n"/>
+      <c r="H12" s="14">
+        <f>IF(G12="","",C12/G12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n"/>
+      <c r="B13" s="36" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="9">
+        <f>IF(C13="","",(C13-D13)/C13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="38" t="n"/>
+      <c r="G13" s="38" t="n"/>
+      <c r="H13" s="14">
+        <f>IF(G13="","",C13/G13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n"/>
+      <c r="B14" s="36" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="9">
+        <f>IF(C14="","",(C14-D14)/C14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="38" t="n"/>
+      <c r="G14" s="38" t="n"/>
+      <c r="H14" s="14">
+        <f>IF(G14="","",C14/G14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n"/>
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="9">
+        <f>IF(C15="","",(C15-D15)/C15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="38" t="n"/>
+      <c r="G15" s="38" t="n"/>
+      <c r="H15" s="14">
+        <f>IF(G15="","",C15/G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="36" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="9">
+        <f>IF(C16="","",(C16-D16)/C16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="38" t="n"/>
+      <c r="G16" s="38" t="n"/>
+      <c r="H16" s="14">
+        <f>IF(G16="","",C16/G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n"/>
+      <c r="B17" s="36" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="9">
+        <f>IF(C17="","",(C17-D17)/C17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="38" t="n"/>
+      <c r="G17" s="38" t="n"/>
+      <c r="H17" s="14">
+        <f>IF(G17="","",C17/G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n"/>
+      <c r="B18" s="36" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="9">
+        <f>IF(C18="","",(C18-D18)/C18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="38" t="n"/>
+      <c r="G18" s="38" t="n"/>
+      <c r="H18" s="14">
+        <f>IF(G18="","",C18/G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n"/>
+      <c r="B19" s="36" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="9">
+        <f>IF(C19="","",(C19-D19)/C19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="38" t="n"/>
+      <c r="G19" s="38" t="n"/>
+      <c r="H19" s="14">
+        <f>IF(G19="","",C19/G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="36" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="9">
+        <f>IF(C20="","",(C20-D20)/C20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="38" t="n"/>
+      <c r="G20" s="38" t="n"/>
+      <c r="H20" s="14">
+        <f>IF(G20="","",C20/G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>PRODUCT PERFORMANCE (monthly)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Units Sold (month)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Revenue (£)</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>COGS (£)</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Net Margin (%)</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n"/>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="9">
+        <f>IF(C24="","",(C24-D24)/C24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="9">
+        <f>IF(C25="","",(C25-D25)/C25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="9">
+        <f>IF(C26="","",(C26-D26)/C26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="16" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="9">
+        <f>IF(C27="","",(C27-D27)/C27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="9">
+        <f>IF(C28="","",(C28-D28)/C28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="9">
+        <f>IF(C29="","",(C29-D29)/C29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n"/>
+      <c r="B30" s="16" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="9">
+        <f>IF(C30="","",(C30-D30)/C30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n"/>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="9">
+        <f>IF(C31="","",(C31-D31)/C31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="16" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="n"/>
+      <c r="B32" s="16" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+      <c r="E32" s="9">
+        <f>IF(C32="","",(C32-D32)/C32)</f>
+        <v/>
+      </c>
+      <c r="F32" s="16" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="n"/>
+      <c r="B33" s="16" t="n"/>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="9">
+        <f>IF(C33="","",(C33-D33)/C33)</f>
+        <v/>
+      </c>
+      <c r="F33" s="16" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="n"/>
+      <c r="B34" s="16" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="9">
+        <f>IF(C34="","",(C34-D34)/C34)</f>
+        <v/>
+      </c>
+      <c r="F34" s="16" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="n"/>
+      <c r="B35" s="16" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="9">
+        <f>IF(C35="","",(C35-D35)/C35)</f>
+        <v/>
+      </c>
+      <c r="F35" s="16" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="n"/>
+      <c r="B36" s="16" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="9">
+        <f>IF(C36="","",(C36-D36)/C36)</f>
+        <v/>
+      </c>
+      <c r="F36" s="16" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="n"/>
+      <c r="B37" s="16" t="n"/>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="9">
+        <f>IF(C37="","",(C37-D37)/C37)</f>
+        <v/>
+      </c>
+      <c r="F37" s="16" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="n"/>
+      <c r="B38" s="16" t="n"/>
+      <c r="C38" s="13" t="n"/>
+      <c r="D38" s="13" t="n"/>
+      <c r="E38" s="9">
+        <f>IF(C38="","",(C38-D38)/C38)</f>
+        <v/>
+      </c>
+      <c r="F38" s="16" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="n"/>
+      <c r="B39" s="16" t="n"/>
+      <c r="C39" s="13" t="n"/>
+      <c r="D39" s="13" t="n"/>
+      <c r="E39" s="9">
+        <f>IF(C39="","",(C39-D39)/C39)</f>
+        <v/>
+      </c>
+      <c r="F39" s="16" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="n"/>
+      <c r="B40" s="16" t="n"/>
+      <c r="C40" s="13" t="n"/>
+      <c r="D40" s="13" t="n"/>
+      <c r="E40" s="9">
+        <f>IF(C40="","",(C40-D40)/C40)</f>
+        <v/>
+      </c>
+      <c r="F40" s="16" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="n"/>
+      <c r="B41" s="16" t="n"/>
+      <c r="C41" s="13" t="n"/>
+      <c r="D41" s="13" t="n"/>
+      <c r="E41" s="9">
+        <f>IF(C41="","",(C41-D41)/C41)</f>
+        <v/>
+      </c>
+      <c r="F41" s="16" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="n"/>
+      <c r="B42" s="16" t="n"/>
+      <c r="C42" s="13" t="n"/>
+      <c r="D42" s="13" t="n"/>
+      <c r="E42" s="9">
+        <f>IF(C42="","",(C42-D42)/C42)</f>
+        <v/>
+      </c>
+      <c r="F42" s="16" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="n"/>
+      <c r="B43" s="16" t="n"/>
+      <c r="C43" s="13" t="n"/>
+      <c r="D43" s="13" t="n"/>
+      <c r="E43" s="9">
+        <f>IF(C43="","",(C43-D43)/C43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>MONTHLY REVIEW GATE — answer before making changes</t>
+        </is>
+      </c>
+      <c r="B45" s="27" t="n"/>
+      <c r="C45" s="27" t="n"/>
+      <c r="D45" s="27" t="n"/>
+      <c r="E45" s="27" t="n"/>
+      <c r="F45" s="27" t="n"/>
+      <c r="G45" s="27" t="n"/>
+      <c r="H45" s="27" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="18" t="inlineStr">
+        <is>
+          <t>OBSERVE</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>What does the data say?</t>
+        </is>
+      </c>
+      <c r="D46" s="24" t="inlineStr">
+        <is>
+          <t>Which sites are above/below target? Which products moved? Which didn't?</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="inlineStr">
+        <is>
+          <t>ORIENT</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>What does this mean?</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="inlineStr">
+        <is>
+          <t>Is a low-performing site a bad location or bad product mix? Is a top seller genuinely popular or just the only option?</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="inlineStr">
+        <is>
+          <t>DECIDE</t>
+        </is>
+      </c>
+      <c r="B48" s="18" t="inlineStr">
+        <is>
+          <t>What will you change?</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="inlineStr">
+        <is>
+          <t>Add/drop products, adjust prices, change visit frequency, drop/add sites. One change at a time — otherwise you can't tell what worked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>Do it. Log it.</t>
+        </is>
+      </c>
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t>Record changes in Methods table on Operations Log. Set a review date. Don't change again until you have 4 weeks of data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>PROTECT</t>
+        </is>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>What could go wrong?</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="inlineStr">
+        <is>
+          <t>Will this change break something? Customer complaint risk? Stock-out risk? Cost increase?</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>KEY RULE: One change at a time. Wait 4 weeks. Then measure.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="H6:H20">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
+      <formula>15</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
+      <formula>30</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="G24:G54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list" type="list">
+      <formula1>"Keep,Increase stock,Reduce stock,Replace,Test new price,Drop"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: add Territory Planner with 14 M25 corridor estates
Researched industrial estates and business parks along the M25 corridor.
Key insight: inner London has too many corner shops for vending to work
(captive audience assumption fails). M25 corridor estates are food deserts
where workers are genuinely captive.

Tier 1 targets (6):
- Park Royal (52,000 workers, largest in London)
- Manor Royal, Crawley (30,000 workers, largest UK industrial BID)
- Slough Trading Estate (13,000 workers)
- Brimsdown, Enfield (7,500 workers, 2nd largest London estate)
- DP World London Gateway (24/7 port, extremely isolated)
- Crossways Business Park, Dartford (direct M25 J1a)

Tier 2 (5): Prologis Park, Watford BP, London Medway, Greenford, Erith
Tier 3 (3): Stockley Park, Croxley Park, Beddington

Green/yellow row colour coding by tier. Filterable.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TheSnackChoice_London_Research.xlsx
+++ b/TheSnackChoice_London_Research.xlsx
@@ -14,13 +14,15 @@
     <sheet name="Competitor Analysis" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Startup Costs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Micro-Market Costs" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Location Tracker" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Weekly P&amp;L" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Operations Log" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Performance Review" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Territory Planner" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Location Tracker" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Weekly P&amp;L" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Operations Log" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Performance Review" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Product Catalog'!$A$1:$N$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Territory Planner'!$A$1:$M$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -93,7 +95,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +126,18 @@
         <bgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -143,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,6 +189,10 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -942,6 +960,421 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Machine ID:</t>
+        </is>
+      </c>
+      <c r="B1" s="19" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Location:</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Week Commencing:</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Cash Revenue (£)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Card Revenue (£)</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Total Revenue (£)</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Units Sold (Cash)</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Units Sold (Card)</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Total Units</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Avg Vend Price (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="n"/>
+      <c r="C6" s="34" t="n"/>
+      <c r="D6" s="14">
+        <f>B6+C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6">
+        <f>E6+F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="14">
+        <f>IF(G6=0,"",D6/G6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B7" s="34" t="n"/>
+      <c r="C7" s="34" t="n"/>
+      <c r="D7" s="14">
+        <f>B7+C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7">
+        <f>E7+F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="14">
+        <f>IF(G7=0,"",D7/G7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="n"/>
+      <c r="C8" s="34" t="n"/>
+      <c r="D8" s="14">
+        <f>B8+C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8">
+        <f>E8+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="14">
+        <f>IF(G8=0,"",D8/G8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="n"/>
+      <c r="C9" s="34" t="n"/>
+      <c r="D9" s="14">
+        <f>B9+C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9">
+        <f>E9+F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="14">
+        <f>IF(G9=0,"",D9/G9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B10" s="34" t="n"/>
+      <c r="C10" s="34" t="n"/>
+      <c r="D10" s="14">
+        <f>B10+C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10">
+        <f>E10+F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="14">
+        <f>IF(G10=0,"",D10/G10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="n"/>
+      <c r="C11" s="34" t="n"/>
+      <c r="D11" s="14">
+        <f>B11+C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11">
+        <f>E11+F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="14">
+        <f>IF(G11=0,"",D11/G11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="n"/>
+      <c r="C12" s="34" t="n"/>
+      <c r="D12" s="14">
+        <f>B12+C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12">
+        <f>E12+F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="14">
+        <f>IF(G12=0,"",D12/G12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>WEEK TOTAL</t>
+        </is>
+      </c>
+      <c r="B13" s="35">
+        <f>SUM(B6:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="35">
+        <f>SUM(C6:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="35">
+        <f>SUM(D6:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="18">
+        <f>SUM(E6:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
+        <f>SUM(F6:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="18">
+        <f>SUM(G6:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="35">
+        <f>IF(G13=0,"",D13/G13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>COSTS</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Amount (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Stock Purchased</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Card Processing Fees</t>
+        </is>
+      </c>
+      <c r="B17" s="37">
+        <f>SUM(C6:C12)*0.029</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Nayax Monthly (pro-rata weekly)</t>
+        </is>
+      </c>
+      <c r="B18" s="37">
+        <f>10/4.33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>Site Rent (pro-rata weekly)</t>
+        </is>
+      </c>
+      <c r="B19" s="36" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Travel/Fuel</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Total Costs</t>
+        </is>
+      </c>
+      <c r="B22" s="38">
+        <f>SUM(B16:B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>WEEKLY SUMMARY</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B25" s="35">
+        <f>D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Total Costs</t>
+        </is>
+      </c>
+      <c r="B26" s="35">
+        <f>B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Net Profit</t>
+        </is>
+      </c>
+      <c r="B27" s="35">
+        <f>B25-B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Gross Margin %</t>
+        </is>
+      </c>
+      <c r="B28" s="39">
+        <f>IF(B25=0,"",(B25-B16)/B25)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1011,188 +1444,188 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="36" t="n"/>
+      <c r="A3" s="40" t="n"/>
       <c r="B3" s="16" t="n"/>
       <c r="C3" s="16" t="n"/>
       <c r="D3" s="16" t="n"/>
-      <c r="E3" s="37" t="n"/>
-      <c r="F3" s="38" t="n"/>
+      <c r="E3" s="41" t="n"/>
+      <c r="F3" s="42" t="n"/>
       <c r="G3" s="16" t="n"/>
       <c r="H3" s="16" t="n"/>
       <c r="I3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="n"/>
+      <c r="A4" s="40" t="n"/>
       <c r="B4" s="16" t="n"/>
       <c r="C4" s="16" t="n"/>
       <c r="D4" s="16" t="n"/>
-      <c r="E4" s="37" t="n"/>
-      <c r="F4" s="38" t="n"/>
+      <c r="E4" s="41" t="n"/>
+      <c r="F4" s="42" t="n"/>
       <c r="G4" s="16" t="n"/>
       <c r="H4" s="16" t="n"/>
       <c r="I4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="n"/>
+      <c r="A5" s="40" t="n"/>
       <c r="B5" s="16" t="n"/>
       <c r="C5" s="16" t="n"/>
       <c r="D5" s="16" t="n"/>
-      <c r="E5" s="37" t="n"/>
-      <c r="F5" s="38" t="n"/>
+      <c r="E5" s="41" t="n"/>
+      <c r="F5" s="42" t="n"/>
       <c r="G5" s="16" t="n"/>
       <c r="H5" s="16" t="n"/>
       <c r="I5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="n"/>
+      <c r="A6" s="40" t="n"/>
       <c r="B6" s="16" t="n"/>
       <c r="C6" s="16" t="n"/>
       <c r="D6" s="16" t="n"/>
-      <c r="E6" s="37" t="n"/>
-      <c r="F6" s="38" t="n"/>
+      <c r="E6" s="41" t="n"/>
+      <c r="F6" s="42" t="n"/>
       <c r="G6" s="16" t="n"/>
       <c r="H6" s="16" t="n"/>
       <c r="I6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="n"/>
+      <c r="A7" s="40" t="n"/>
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="37" t="n"/>
-      <c r="F7" s="38" t="n"/>
+      <c r="E7" s="41" t="n"/>
+      <c r="F7" s="42" t="n"/>
       <c r="G7" s="16" t="n"/>
       <c r="H7" s="16" t="n"/>
       <c r="I7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="n"/>
+      <c r="A8" s="40" t="n"/>
       <c r="B8" s="16" t="n"/>
       <c r="C8" s="16" t="n"/>
       <c r="D8" s="16" t="n"/>
-      <c r="E8" s="37" t="n"/>
-      <c r="F8" s="38" t="n"/>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="42" t="n"/>
       <c r="G8" s="16" t="n"/>
       <c r="H8" s="16" t="n"/>
       <c r="I8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="n"/>
+      <c r="A9" s="40" t="n"/>
       <c r="B9" s="16" t="n"/>
       <c r="C9" s="16" t="n"/>
       <c r="D9" s="16" t="n"/>
-      <c r="E9" s="37" t="n"/>
-      <c r="F9" s="38" t="n"/>
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="42" t="n"/>
       <c r="G9" s="16" t="n"/>
       <c r="H9" s="16" t="n"/>
       <c r="I9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="n"/>
+      <c r="A10" s="40" t="n"/>
       <c r="B10" s="16" t="n"/>
       <c r="C10" s="16" t="n"/>
       <c r="D10" s="16" t="n"/>
-      <c r="E10" s="37" t="n"/>
-      <c r="F10" s="38" t="n"/>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="42" t="n"/>
       <c r="G10" s="16" t="n"/>
       <c r="H10" s="16" t="n"/>
       <c r="I10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="n"/>
+      <c r="A11" s="40" t="n"/>
       <c r="B11" s="16" t="n"/>
       <c r="C11" s="16" t="n"/>
       <c r="D11" s="16" t="n"/>
-      <c r="E11" s="37" t="n"/>
-      <c r="F11" s="38" t="n"/>
+      <c r="E11" s="41" t="n"/>
+      <c r="F11" s="42" t="n"/>
       <c r="G11" s="16" t="n"/>
       <c r="H11" s="16" t="n"/>
       <c r="I11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="n"/>
+      <c r="A12" s="40" t="n"/>
       <c r="B12" s="16" t="n"/>
       <c r="C12" s="16" t="n"/>
       <c r="D12" s="16" t="n"/>
-      <c r="E12" s="37" t="n"/>
-      <c r="F12" s="38" t="n"/>
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="42" t="n"/>
       <c r="G12" s="16" t="n"/>
       <c r="H12" s="16" t="n"/>
       <c r="I12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="n"/>
+      <c r="A13" s="40" t="n"/>
       <c r="B13" s="16" t="n"/>
       <c r="C13" s="16" t="n"/>
       <c r="D13" s="16" t="n"/>
-      <c r="E13" s="37" t="n"/>
-      <c r="F13" s="38" t="n"/>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="42" t="n"/>
       <c r="G13" s="16" t="n"/>
       <c r="H13" s="16" t="n"/>
       <c r="I13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="n"/>
+      <c r="A14" s="40" t="n"/>
       <c r="B14" s="16" t="n"/>
       <c r="C14" s="16" t="n"/>
       <c r="D14" s="16" t="n"/>
-      <c r="E14" s="37" t="n"/>
-      <c r="F14" s="38" t="n"/>
+      <c r="E14" s="41" t="n"/>
+      <c r="F14" s="42" t="n"/>
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
       <c r="I14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="n"/>
+      <c r="A15" s="40" t="n"/>
       <c r="B15" s="16" t="n"/>
       <c r="C15" s="16" t="n"/>
       <c r="D15" s="16" t="n"/>
-      <c r="E15" s="37" t="n"/>
-      <c r="F15" s="38" t="n"/>
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="42" t="n"/>
       <c r="G15" s="16" t="n"/>
       <c r="H15" s="16" t="n"/>
       <c r="I15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="n"/>
+      <c r="A16" s="40" t="n"/>
       <c r="B16" s="16" t="n"/>
       <c r="C16" s="16" t="n"/>
       <c r="D16" s="16" t="n"/>
-      <c r="E16" s="37" t="n"/>
-      <c r="F16" s="38" t="n"/>
+      <c r="E16" s="41" t="n"/>
+      <c r="F16" s="42" t="n"/>
       <c r="G16" s="16" t="n"/>
       <c r="H16" s="16" t="n"/>
       <c r="I16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="36" t="n"/>
+      <c r="A17" s="40" t="n"/>
       <c r="B17" s="16" t="n"/>
       <c r="C17" s="16" t="n"/>
       <c r="D17" s="16" t="n"/>
-      <c r="E17" s="37" t="n"/>
-      <c r="F17" s="38" t="n"/>
+      <c r="E17" s="41" t="n"/>
+      <c r="F17" s="42" t="n"/>
       <c r="G17" s="16" t="n"/>
       <c r="H17" s="16" t="n"/>
       <c r="I17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="36" t="n"/>
+      <c r="A18" s="40" t="n"/>
       <c r="B18" s="16" t="n"/>
       <c r="C18" s="16" t="n"/>
       <c r="D18" s="16" t="n"/>
-      <c r="E18" s="37" t="n"/>
-      <c r="F18" s="38" t="n"/>
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="42" t="n"/>
       <c r="G18" s="16" t="n"/>
       <c r="H18" s="16" t="n"/>
       <c r="I18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="36" t="n"/>
+      <c r="A19" s="40" t="n"/>
       <c r="B19" s="16" t="n"/>
       <c r="C19" s="16" t="n"/>
       <c r="D19" s="16" t="n"/>
-      <c r="E19" s="37" t="n"/>
-      <c r="F19" s="38" t="n"/>
+      <c r="E19" s="41" t="n"/>
+      <c r="F19" s="42" t="n"/>
       <c r="G19" s="16" t="n"/>
       <c r="H19" s="16" t="n"/>
       <c r="I19" s="13" t="n"/>
@@ -1252,7 +1685,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="36" t="n"/>
+      <c r="A24" s="40" t="n"/>
       <c r="B24" s="16" t="n"/>
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="16" t="n"/>
@@ -1263,7 +1696,7 @@
       <c r="I24" s="16" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="36" t="n"/>
+      <c r="A25" s="40" t="n"/>
       <c r="B25" s="16" t="n"/>
       <c r="C25" s="16" t="n"/>
       <c r="D25" s="16" t="n"/>
@@ -1274,7 +1707,7 @@
       <c r="I25" s="16" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="36" t="n"/>
+      <c r="A26" s="40" t="n"/>
       <c r="B26" s="16" t="n"/>
       <c r="C26" s="16" t="n"/>
       <c r="D26" s="16" t="n"/>
@@ -1285,7 +1718,7 @@
       <c r="I26" s="16" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="36" t="n"/>
+      <c r="A27" s="40" t="n"/>
       <c r="B27" s="16" t="n"/>
       <c r="C27" s="16" t="n"/>
       <c r="D27" s="16" t="n"/>
@@ -1296,7 +1729,7 @@
       <c r="I27" s="16" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="36" t="n"/>
+      <c r="A28" s="40" t="n"/>
       <c r="B28" s="16" t="n"/>
       <c r="C28" s="16" t="n"/>
       <c r="D28" s="16" t="n"/>
@@ -1307,7 +1740,7 @@
       <c r="I28" s="16" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="36" t="n"/>
+      <c r="A29" s="40" t="n"/>
       <c r="B29" s="16" t="n"/>
       <c r="C29" s="16" t="n"/>
       <c r="D29" s="16" t="n"/>
@@ -1318,7 +1751,7 @@
       <c r="I29" s="16" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="36" t="n"/>
+      <c r="A30" s="40" t="n"/>
       <c r="B30" s="16" t="n"/>
       <c r="C30" s="16" t="n"/>
       <c r="D30" s="16" t="n"/>
@@ -1329,7 +1762,7 @@
       <c r="I30" s="16" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="36" t="n"/>
+      <c r="A31" s="40" t="n"/>
       <c r="B31" s="16" t="n"/>
       <c r="C31" s="16" t="n"/>
       <c r="D31" s="16" t="n"/>
@@ -1340,7 +1773,7 @@
       <c r="I31" s="16" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="36" t="n"/>
+      <c r="A32" s="40" t="n"/>
       <c r="B32" s="16" t="n"/>
       <c r="C32" s="16" t="n"/>
       <c r="D32" s="16" t="n"/>
@@ -1351,7 +1784,7 @@
       <c r="I32" s="16" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="36" t="n"/>
+      <c r="A33" s="40" t="n"/>
       <c r="B33" s="16" t="n"/>
       <c r="C33" s="16" t="n"/>
       <c r="D33" s="16" t="n"/>
@@ -1476,7 +1909,7 @@
           <t>JIT (buy morning of restock)</t>
         </is>
       </c>
-      <c r="C45" s="39" t="inlineStr"/>
+      <c r="C45" s="43" t="inlineStr"/>
       <c r="D45" s="24" t="inlineStr">
         <is>
           <t>Switch to bulk when 5+ machines</t>
@@ -1494,7 +1927,7 @@
           <t>2x/week per machine</t>
         </is>
       </c>
-      <c r="C46" s="39" t="inlineStr"/>
+      <c r="C46" s="43" t="inlineStr"/>
       <c r="D46" s="24" t="inlineStr">
         <is>
           <t>Adjust per site based on Nayax data</t>
@@ -1512,7 +1945,7 @@
           <t>Monthly — swap bottom 3 sellers</t>
         </is>
       </c>
-      <c r="C47" s="39" t="inlineStr"/>
+      <c r="C47" s="43" t="inlineStr"/>
       <c r="D47" s="24" t="inlineStr">
         <is>
           <t>Track via Weekly P&amp;L</t>
@@ -1530,7 +1963,7 @@
           <t>60%+ net margin target</t>
         </is>
       </c>
-      <c r="C48" s="39" t="inlineStr"/>
+      <c r="C48" s="43" t="inlineStr"/>
       <c r="D48" s="24" t="inlineStr">
         <is>
           <t>Premium sites can go higher</t>
@@ -1548,7 +1981,7 @@
           <t>30% net minimum to stock</t>
         </is>
       </c>
-      <c r="C49" s="39" t="inlineStr"/>
+      <c r="C49" s="43" t="inlineStr"/>
       <c r="D49" s="24" t="inlineStr">
         <is>
           <t>Below this, product isn't worth the slot</t>
@@ -1566,7 +1999,7 @@
           <t>30 min per machine</t>
         </is>
       </c>
-      <c r="C50" s="39" t="inlineStr"/>
+      <c r="C50" s="43" t="inlineStr"/>
       <c r="D50" s="24" t="inlineStr">
         <is>
           <t>Including travel, restock, clean</t>
@@ -1584,7 +2017,7 @@
           <t>5% — investigate above this</t>
         </is>
       </c>
-      <c r="C51" s="39" t="inlineStr"/>
+      <c r="C51" s="43" t="inlineStr"/>
       <c r="D51" s="24" t="inlineStr">
         <is>
           <t>Camera or format change if persistent</t>
@@ -1610,7 +2043,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1637,7 +2070,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="40" t="inlineStr">
+      <c r="A2" s="44" t="inlineStr">
         <is>
           <t>Fill weekly. Review monthly. Beliefs and methods evolve from what you see here.</t>
         </is>
@@ -1701,15 +2134,15 @@
     </row>
     <row r="6">
       <c r="A6" s="16" t="n"/>
-      <c r="B6" s="36" t="n"/>
+      <c r="B6" s="40" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="9">
         <f>IF(C6="","",(C6-D6)/C6)</f>
         <v/>
       </c>
-      <c r="F6" s="38" t="n"/>
-      <c r="G6" s="38" t="n"/>
+      <c r="F6" s="42" t="n"/>
+      <c r="G6" s="42" t="n"/>
       <c r="H6" s="14">
         <f>IF(G6="","",C6/G6)</f>
         <v/>
@@ -1717,15 +2150,15 @@
     </row>
     <row r="7">
       <c r="A7" s="16" t="n"/>
-      <c r="B7" s="36" t="n"/>
+      <c r="B7" s="40" t="n"/>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="9">
         <f>IF(C7="","",(C7-D7)/C7)</f>
         <v/>
       </c>
-      <c r="F7" s="38" t="n"/>
-      <c r="G7" s="38" t="n"/>
+      <c r="F7" s="42" t="n"/>
+      <c r="G7" s="42" t="n"/>
       <c r="H7" s="14">
         <f>IF(G7="","",C7/G7)</f>
         <v/>
@@ -1733,15 +2166,15 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="n"/>
-      <c r="B8" s="36" t="n"/>
+      <c r="B8" s="40" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="9">
         <f>IF(C8="","",(C8-D8)/C8)</f>
         <v/>
       </c>
-      <c r="F8" s="38" t="n"/>
-      <c r="G8" s="38" t="n"/>
+      <c r="F8" s="42" t="n"/>
+      <c r="G8" s="42" t="n"/>
       <c r="H8" s="14">
         <f>IF(G8="","",C8/G8)</f>
         <v/>
@@ -1749,15 +2182,15 @@
     </row>
     <row r="9">
       <c r="A9" s="16" t="n"/>
-      <c r="B9" s="36" t="n"/>
+      <c r="B9" s="40" t="n"/>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="9">
         <f>IF(C9="","",(C9-D9)/C9)</f>
         <v/>
       </c>
-      <c r="F9" s="38" t="n"/>
-      <c r="G9" s="38" t="n"/>
+      <c r="F9" s="42" t="n"/>
+      <c r="G9" s="42" t="n"/>
       <c r="H9" s="14">
         <f>IF(G9="","",C9/G9)</f>
         <v/>
@@ -1765,15 +2198,15 @@
     </row>
     <row r="10">
       <c r="A10" s="16" t="n"/>
-      <c r="B10" s="36" t="n"/>
+      <c r="B10" s="40" t="n"/>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="9">
         <f>IF(C10="","",(C10-D10)/C10)</f>
         <v/>
       </c>
-      <c r="F10" s="38" t="n"/>
-      <c r="G10" s="38" t="n"/>
+      <c r="F10" s="42" t="n"/>
+      <c r="G10" s="42" t="n"/>
       <c r="H10" s="14">
         <f>IF(G10="","",C10/G10)</f>
         <v/>
@@ -1781,15 +2214,15 @@
     </row>
     <row r="11">
       <c r="A11" s="16" t="n"/>
-      <c r="B11" s="36" t="n"/>
+      <c r="B11" s="40" t="n"/>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="9">
         <f>IF(C11="","",(C11-D11)/C11)</f>
         <v/>
       </c>
-      <c r="F11" s="38" t="n"/>
-      <c r="G11" s="38" t="n"/>
+      <c r="F11" s="42" t="n"/>
+      <c r="G11" s="42" t="n"/>
       <c r="H11" s="14">
         <f>IF(G11="","",C11/G11)</f>
         <v/>
@@ -1797,15 +2230,15 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="n"/>
-      <c r="B12" s="36" t="n"/>
+      <c r="B12" s="40" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="9">
         <f>IF(C12="","",(C12-D12)/C12)</f>
         <v/>
       </c>
-      <c r="F12" s="38" t="n"/>
-      <c r="G12" s="38" t="n"/>
+      <c r="F12" s="42" t="n"/>
+      <c r="G12" s="42" t="n"/>
       <c r="H12" s="14">
         <f>IF(G12="","",C12/G12)</f>
         <v/>
@@ -1813,15 +2246,15 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="n"/>
-      <c r="B13" s="36" t="n"/>
+      <c r="B13" s="40" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="9">
         <f>IF(C13="","",(C13-D13)/C13)</f>
         <v/>
       </c>
-      <c r="F13" s="38" t="n"/>
-      <c r="G13" s="38" t="n"/>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="42" t="n"/>
       <c r="H13" s="14">
         <f>IF(G13="","",C13/G13)</f>
         <v/>
@@ -1829,15 +2262,15 @@
     </row>
     <row r="14">
       <c r="A14" s="16" t="n"/>
-      <c r="B14" s="36" t="n"/>
+      <c r="B14" s="40" t="n"/>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="9">
         <f>IF(C14="","",(C14-D14)/C14)</f>
         <v/>
       </c>
-      <c r="F14" s="38" t="n"/>
-      <c r="G14" s="38" t="n"/>
+      <c r="F14" s="42" t="n"/>
+      <c r="G14" s="42" t="n"/>
       <c r="H14" s="14">
         <f>IF(G14="","",C14/G14)</f>
         <v/>
@@ -1845,15 +2278,15 @@
     </row>
     <row r="15">
       <c r="A15" s="16" t="n"/>
-      <c r="B15" s="36" t="n"/>
+      <c r="B15" s="40" t="n"/>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="9">
         <f>IF(C15="","",(C15-D15)/C15)</f>
         <v/>
       </c>
-      <c r="F15" s="38" t="n"/>
-      <c r="G15" s="38" t="n"/>
+      <c r="F15" s="42" t="n"/>
+      <c r="G15" s="42" t="n"/>
       <c r="H15" s="14">
         <f>IF(G15="","",C15/G15)</f>
         <v/>
@@ -1861,15 +2294,15 @@
     </row>
     <row r="16">
       <c r="A16" s="16" t="n"/>
-      <c r="B16" s="36" t="n"/>
+      <c r="B16" s="40" t="n"/>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="9">
         <f>IF(C16="","",(C16-D16)/C16)</f>
         <v/>
       </c>
-      <c r="F16" s="38" t="n"/>
-      <c r="G16" s="38" t="n"/>
+      <c r="F16" s="42" t="n"/>
+      <c r="G16" s="42" t="n"/>
       <c r="H16" s="14">
         <f>IF(G16="","",C16/G16)</f>
         <v/>
@@ -1877,15 +2310,15 @@
     </row>
     <row r="17">
       <c r="A17" s="16" t="n"/>
-      <c r="B17" s="36" t="n"/>
+      <c r="B17" s="40" t="n"/>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="9">
         <f>IF(C17="","",(C17-D17)/C17)</f>
         <v/>
       </c>
-      <c r="F17" s="38" t="n"/>
-      <c r="G17" s="38" t="n"/>
+      <c r="F17" s="42" t="n"/>
+      <c r="G17" s="42" t="n"/>
       <c r="H17" s="14">
         <f>IF(G17="","",C17/G17)</f>
         <v/>
@@ -1893,15 +2326,15 @@
     </row>
     <row r="18">
       <c r="A18" s="16" t="n"/>
-      <c r="B18" s="36" t="n"/>
+      <c r="B18" s="40" t="n"/>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="9">
         <f>IF(C18="","",(C18-D18)/C18)</f>
         <v/>
       </c>
-      <c r="F18" s="38" t="n"/>
-      <c r="G18" s="38" t="n"/>
+      <c r="F18" s="42" t="n"/>
+      <c r="G18" s="42" t="n"/>
       <c r="H18" s="14">
         <f>IF(G18="","",C18/G18)</f>
         <v/>
@@ -1909,15 +2342,15 @@
     </row>
     <row r="19">
       <c r="A19" s="16" t="n"/>
-      <c r="B19" s="36" t="n"/>
+      <c r="B19" s="40" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="9">
         <f>IF(C19="","",(C19-D19)/C19)</f>
         <v/>
       </c>
-      <c r="F19" s="38" t="n"/>
-      <c r="G19" s="38" t="n"/>
+      <c r="F19" s="42" t="n"/>
+      <c r="G19" s="42" t="n"/>
       <c r="H19" s="14">
         <f>IF(G19="","",C19/G19)</f>
         <v/>
@@ -1925,15 +2358,15 @@
     </row>
     <row r="20">
       <c r="A20" s="16" t="n"/>
-      <c r="B20" s="36" t="n"/>
+      <c r="B20" s="40" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="9">
         <f>IF(C20="","",(C20-D20)/C20)</f>
         <v/>
       </c>
-      <c r="F20" s="38" t="n"/>
-      <c r="G20" s="38" t="n"/>
+      <c r="F20" s="42" t="n"/>
+      <c r="G20" s="42" t="n"/>
       <c r="H20" s="14">
         <f>IF(G20="","",C20/G20)</f>
         <v/>
@@ -2315,7 +2748,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="41" t="inlineStr">
+      <c r="A52" s="45" t="inlineStr">
         <is>
           <t>KEY RULE: One change at a time. Wait 4 weeks. Then measure.</t>
         </is>
@@ -10656,6 +11089,948 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Estate/Park Name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Postcode</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>M25 Junction</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Size (acres)</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Est. Workers</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Businesses</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Business Types</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Anchor Tenants</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Food Access</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
+        <is>
+          <t>Vending Score (1-10)</t>
+        </is>
+      </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="M1" s="11" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Park Royal</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="inlineStr">
+        <is>
+          <t>NW10 / W3, Ealing &amp; Brent</t>
+        </is>
+      </c>
+      <c r="C2" s="29" t="inlineStr">
+        <is>
+          <t>NW10</t>
+        </is>
+      </c>
+      <c r="D2" s="29" t="inlineStr">
+        <is>
+          <t>Via A40/North Circular</t>
+        </is>
+      </c>
+      <c r="E2" s="29" t="n">
+        <v>1443</v>
+      </c>
+      <c r="F2" s="29" t="inlineStr">
+        <is>
+          <t>36,000-52,000</t>
+        </is>
+      </c>
+      <c r="G2" s="29" t="inlineStr">
+        <is>
+          <t>1,700+</t>
+        </is>
+      </c>
+      <c r="H2" s="29" t="inlineStr">
+        <is>
+          <t>Food manufacturing, logistics, light industrial, creative</t>
+        </is>
+      </c>
+      <c r="I2" s="29" t="inlineStr">
+        <is>
+          <t>Diageo, Coca-Cola, Sky, Disney, British Airways</t>
+        </is>
+      </c>
+      <c r="J2" s="29" t="inlineStr">
+        <is>
+          <t>Dispersed, many areas with none. Mobile catering vans.</t>
+        </is>
+      </c>
+      <c r="K2" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="29" t="inlineStr">
+        <is>
+          <t>Largest industrial estate in London. 500+ food manufacturers = shift workers. Fragmented ownership = many underserved pockets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Manor Royal</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>Crawley, West Sussex</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
+        <is>
+          <t>RH10</t>
+        </is>
+      </c>
+      <c r="D3" s="29" t="inlineStr">
+        <is>
+          <t>M23 J10 (south of M25)</t>
+        </is>
+      </c>
+      <c r="E3" s="29" t="n">
+        <v>540</v>
+      </c>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>30,000+</t>
+        </is>
+      </c>
+      <c r="G3" s="29" t="inlineStr">
+        <is>
+          <t>600+</t>
+        </is>
+      </c>
+      <c r="H3" s="29" t="inlineStr">
+        <is>
+          <t>Aviation, manufacturing, logistics, pharma, offices</t>
+        </is>
+      </c>
+      <c r="I3" s="29" t="inlineStr">
+        <is>
+          <t>Virgin Atlantic, Thales, Tesco.com, Nestle, Elekta</t>
+        </is>
+      </c>
+      <c r="J3" s="29" t="inlineStr">
+        <is>
+          <t>Bank Precinct has some. Vast areas are 10+ min walk from food.</t>
+        </is>
+      </c>
+      <c r="K3" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="L3" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="29" t="inlineStr">
+        <is>
+          <t>UK's largest industrial BID. Organised management body to approach. £1.7bn GVA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Slough Trading Estate</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>Slough, Berkshire</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t>SL1</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t>M4 J6/J7, M25 J15</t>
+        </is>
+      </c>
+      <c r="E4" s="29" t="n">
+        <v>353</v>
+      </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>~13,000</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>~350</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>Logistics, offices, light manufacturing, R&amp;D, data centres</t>
+        </is>
+      </c>
+      <c r="I4" s="29" t="inlineStr">
+        <is>
+          <t>Mars, Dulux (AkzoNobel)</t>
+        </is>
+      </c>
+      <c r="J4" s="29" t="inlineStr">
+        <is>
+          <t>Some on-estate catering. Peripheral areas remote from shops.</t>
+        </is>
+      </c>
+      <c r="K4" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="L4" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="29" t="inlineStr">
+        <is>
+          <t>SEGRO-owned. 435 units. 24/7 warehouse operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Brimsdown Industrial Estate</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Enfield, North London</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>EN3</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>J25 (~3 miles)</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="n">
+        <v>286</v>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>~7,500</t>
+        </is>
+      </c>
+      <c r="G5" s="29" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
+      </c>
+      <c r="H5" s="29" t="inlineStr">
+        <is>
+          <t>Manufacturing, food production, logistics, chemicals</t>
+        </is>
+      </c>
+      <c r="I5" s="29" t="inlineStr">
+        <is>
+          <t>Johnson Matthey, Warburtons, Greggs, DHL</t>
+        </is>
+      </c>
+      <c r="J5" s="29" t="inlineStr">
+        <is>
+          <t>Very poorly served. Enfield town centre 2 miles away.</t>
+        </is>
+      </c>
+      <c r="K5" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="L5" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="29" t="inlineStr">
+        <is>
+          <t>London's 2nd largest industrial estate. £721m GVA. Multiple sub-estates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>DP World London Gateway</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Stanford-le-Hope, Thurrock</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>SS17</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>A13 to J30/31</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>Growing (1,500+)</t>
+        </is>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>17 facilities</t>
+        </is>
+      </c>
+      <c r="H6" s="29" t="inlineStr">
+        <is>
+          <t>Port logistics, distribution, sorting/fulfilment</t>
+        </is>
+      </c>
+      <c r="I6" s="29" t="inlineStr">
+        <is>
+          <t>UPS, DHL, Curry's</t>
+        </is>
+      </c>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>Extremely isolated. Stanford-le-Hope 2 miles.</t>
+        </is>
+      </c>
+      <c r="K6" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="29" t="inlineStr">
+        <is>
+          <t>24/7 port operations. 9M sq ft logistics park, 50% built. New 10-year expansion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Crossways Business Park</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Dartford, Kent</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>DA2</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>J1a (direct)</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>300</v>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>1,000+</t>
+        </is>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>45+</t>
+        </is>
+      </c>
+      <c r="H7" s="29" t="inlineStr">
+        <is>
+          <t>Logistics, distribution, data centres, food distribution</t>
+        </is>
+      </c>
+      <c r="I7" s="29" t="inlineStr">
+        <is>
+          <t>John Lewis, Kuehne+Nagel, ASDA, DHL, Yodel</t>
+        </is>
+      </c>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>Dartford town centre 3 miles. Limited on-site.</t>
+        </is>
+      </c>
+      <c r="K7" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="L7" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="29" t="inlineStr">
+        <is>
+          <t>3M+ sq ft. Phase 2 adding 318,000 sq ft. 24/7 shift patterns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Prologis Park West London</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>West Drayton, Hillingdon</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UB7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>J15, M4 J4</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>500-2,000 (est.)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6 large units</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Big-box logistics, B8 warehousing</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Major logistics operators (not confirmed)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Zero on-site. 15 min walk to West Drayton station.</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Large logistics warehouses with shift workers. Approach individual occupiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Watford Business Park</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Watford, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>WD18</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>M1 J5 (1.2 miles)</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2,000-5,000 (est.)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>100+</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Mixed industrial/office</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Corona Energy, Kodak</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Some periphery retail. Estate itself is industrial.</t>
+        </is>
+      </c>
+      <c r="K9" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>New £25M development. Growing. Good mix of logistics and office.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>London Medway Commercial Park</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Strood, Kent</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ME2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>A2/M2 corridor</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>115</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>6+ major</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Logistics, distribution</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Amazon, Wincanton, Noatum Logistics</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Limited on-site.</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Goodman-developed. 24/7 distribution operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SEGRO Greenford Central</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Greenford, Ealing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>UB6</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Via A40/M40</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Multi-unit</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Industrial, warehouse, trade counter</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>SEGRO-managed, various SME</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Some high street nearby. Estate itself is industrial.</t>
+        </is>
+      </c>
+      <c r="K11" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Expanding 250,000+ sq ft. Major redevelopment 2027/28.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thames Road / Erith-Belvedere Corridor</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Erith/Crayford, Kent</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DA1/DA8</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>J1a/J2 via A2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1,000+ (est.)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Light industrial, warehousing, trade counter</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Various SME</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Limited. Scattered convenience in residential areas.</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Dense industrial strip. Multiple estates along Thames Road.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Beddington Trading Estate</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CR0</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>J7 (~6 miles)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>500+ (est.)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Multi-unit</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Warehousing, light industrial</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Capital Industrial (landlord)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Purley Way retail 0.5 miles but not walkable (industrial roads).</t>
+        </is>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Workers unlikely to walk to Purley Way during breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>Stockley Park</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>Uxbridge, Hillingdon</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>UB11</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
+          <t>M4 J4, M25 J15</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="n">
+        <v>150</v>
+      </c>
+      <c r="F14" s="31" t="inlineStr">
+        <is>
+          <t>Several thousand</t>
+        </is>
+      </c>
+      <c r="G14" s="31" t="inlineStr">
+        <is>
+          <t>20+ major</t>
+        </is>
+      </c>
+      <c r="H14" s="31" t="inlineStr">
+        <is>
+          <t>Corporate HQ, tech, pharma</t>
+        </is>
+      </c>
+      <c r="I14" s="31" t="inlineStr">
+        <is>
+          <t>Apple, GSK, Canon, Hasbro, Marks &amp; Spencer</t>
+        </is>
+      </c>
+      <c r="J14" s="31" t="inlineStr">
+        <is>
+          <t>On-park amenities at The Square. Premium managed campus.</t>
+        </is>
+      </c>
+      <c r="K14" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="31" t="inlineStr">
+        <is>
+          <t>Premium campus — likely has catering. Opportunity in buildings without canteens. Requires healthy/premium product mix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>Croxley Park</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>Watford, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>WD18</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>M25 corridor</t>
+        </is>
+      </c>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="inlineStr">
+        <is>
+          <t>2,400+</t>
+        </is>
+      </c>
+      <c r="G15" s="31" t="inlineStr">
+        <is>
+          <t>Multi-tenant campus</t>
+        </is>
+      </c>
+      <c r="H15" s="31" t="inlineStr">
+        <is>
+          <t>Corporate offices</t>
+        </is>
+      </c>
+      <c r="I15" s="31" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="J15" s="31" t="inlineStr">
+        <is>
+          <t>Not walkable to town. Shuttle bus to Watford Junction.</t>
+        </is>
+      </c>
+      <c r="K15" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" s="31" t="inlineStr">
+        <is>
+          <t>Managed campus. Check what on-site catering exists.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M20"/>
+  <dataValidations count="1">
+    <dataValidation sqref="L2:L50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -10829,419 +12204,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Machine ID:</t>
-        </is>
-      </c>
-      <c r="B1" s="19" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="18" t="inlineStr">
-        <is>
-          <t>Location:</t>
-        </is>
-      </c>
-      <c r="B2" s="19" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="18" t="inlineStr">
-        <is>
-          <t>Week Commencing:</t>
-        </is>
-      </c>
-      <c r="B3" s="29" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Cash Revenue (£)</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>Card Revenue (£)</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Total Revenue (£)</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>Units Sold (Cash)</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>Units Sold (Card)</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>Total Units</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>Avg Vend Price (£)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="n"/>
-      <c r="C6" s="30" t="n"/>
-      <c r="D6" s="14">
-        <f>B6+C6</f>
-        <v/>
-      </c>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="19" t="n"/>
-      <c r="G6">
-        <f>E6+F6</f>
-        <v/>
-      </c>
-      <c r="H6" s="14">
-        <f>IF(G6=0,"",D6/G6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="n"/>
-      <c r="C7" s="30" t="n"/>
-      <c r="D7" s="14">
-        <f>B7+C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="19" t="n"/>
-      <c r="F7" s="19" t="n"/>
-      <c r="G7">
-        <f>E7+F7</f>
-        <v/>
-      </c>
-      <c r="H7" s="14">
-        <f>IF(G7=0,"",D7/G7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="n"/>
-      <c r="C8" s="30" t="n"/>
-      <c r="D8" s="14">
-        <f>B8+C8</f>
-        <v/>
-      </c>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="19" t="n"/>
-      <c r="G8">
-        <f>E8+F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="14">
-        <f>IF(G8=0,"",D8/G8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="n"/>
-      <c r="C9" s="30" t="n"/>
-      <c r="D9" s="14">
-        <f>B9+C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="19" t="n"/>
-      <c r="F9" s="19" t="n"/>
-      <c r="G9">
-        <f>E9+F9</f>
-        <v/>
-      </c>
-      <c r="H9" s="14">
-        <f>IF(G9=0,"",D9/G9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="n"/>
-      <c r="C10" s="30" t="n"/>
-      <c r="D10" s="14">
-        <f>B10+C10</f>
-        <v/>
-      </c>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10">
-        <f>E10+F10</f>
-        <v/>
-      </c>
-      <c r="H10" s="14">
-        <f>IF(G10=0,"",D10/G10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="n"/>
-      <c r="C11" s="30" t="n"/>
-      <c r="D11" s="14">
-        <f>B11+C11</f>
-        <v/>
-      </c>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11">
-        <f>E11+F11</f>
-        <v/>
-      </c>
-      <c r="H11" s="14">
-        <f>IF(G11=0,"",D11/G11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="n"/>
-      <c r="C12" s="30" t="n"/>
-      <c r="D12" s="14">
-        <f>B12+C12</f>
-        <v/>
-      </c>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12">
-        <f>E12+F12</f>
-        <v/>
-      </c>
-      <c r="H12" s="14">
-        <f>IF(G12=0,"",D12/G12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>WEEK TOTAL</t>
-        </is>
-      </c>
-      <c r="B13" s="31">
-        <f>SUM(B6:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="31">
-        <f>SUM(C6:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="31">
-        <f>SUM(D6:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="18">
-        <f>SUM(E6:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="18">
-        <f>SUM(F6:F12)</f>
-        <v/>
-      </c>
-      <c r="G13" s="18">
-        <f>SUM(G6:G12)</f>
-        <v/>
-      </c>
-      <c r="H13" s="31">
-        <f>IF(G13=0,"",D13/G13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>COSTS</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>Amount (£)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>Stock Purchased</t>
-        </is>
-      </c>
-      <c r="B16" s="32" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>Card Processing Fees</t>
-        </is>
-      </c>
-      <c r="B17" s="33">
-        <f>SUM(C6:C12)*0.029</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="21" t="inlineStr">
-        <is>
-          <t>Nayax Monthly (pro-rata weekly)</t>
-        </is>
-      </c>
-      <c r="B18" s="33">
-        <f>10/4.33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>Site Rent (pro-rata weekly)</t>
-        </is>
-      </c>
-      <c r="B19" s="32" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>Travel/Fuel</t>
-        </is>
-      </c>
-      <c r="B20" s="32" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="21" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B21" s="32" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Total Costs</t>
-        </is>
-      </c>
-      <c r="B22" s="34">
-        <f>SUM(B16:B21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>WEEKLY SUMMARY</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Gross Revenue</t>
-        </is>
-      </c>
-      <c r="B25" s="31">
-        <f>D13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>Total Costs</t>
-        </is>
-      </c>
-      <c r="B26" s="31">
-        <f>B22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Net Profit</t>
-        </is>
-      </c>
-      <c r="B27" s="31">
-        <f>B25-B26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Gross Margin %</t>
-        </is>
-      </c>
-      <c r="B28" s="35">
-        <f>IF(B25=0,"",(B25-B16)/B25)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: food desert analysis via Google Places — 7 estates scouted
Used scout tool to systematically search for food retail within each
estate's industrial zone. Key findings:

CONFIRMED FOOD DESERTS:
- Park Royal: 12 outlets for 52,000 workers (1:4,333). Interior has 3.
- London Gateway: 3 outlets on 1,500 acres. Extremely isolated.

PARTIAL DESERTS:
- Manor Royal: 16 outlets but 3 are snack vans. Western half empty.
- Brimsdown: 7 outlets, western interior has zero food.
- Crossways: Costa only quick option. No grab-and-go.
- Watford BP: 2 on-site, rescued by nearby residential shops.

DOWNGRADED:
- Slough TE: 20 outlets inc Lidl, Iceland, 3 Greggs. Moved to Tier 2.

Territory Planner updated with verified food access data and scores.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TheSnackChoice_London_Research.xlsx
+++ b/TheSnackChoice_London_Research.xlsx
@@ -11984,7 +11984,7 @@
       </c>
       <c r="J2" s="32" t="inlineStr">
         <is>
-          <t>Dispersed, many areas with none. Mobile catering vans.</t>
+          <t>FOOD DESERT. 12 outlets for 52,000 workers (1:4,333). Deep interior has 3 outlets only. Zero food on Minerva Rd, Twyford Abbey area.</t>
         </is>
       </c>
       <c r="K2" s="33" t="n">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="M2" s="32" t="inlineStr">
         <is>
-          <t>Largest industrial estate in London. 500+ food manufacturers = shift workers. Fragmented ownership = many underserved pockets.</t>
+          <t>SCOUT VERIFIED. Largest industrial estate in London. 500+ food manufacturers = shift workers. 3 outlets serve entire interior. Best vending opportunity.</t>
         </is>
       </c>
     </row>
@@ -12045,79 +12045,79 @@
       </c>
       <c r="J3" s="32" t="inlineStr">
         <is>
-          <t>Bank Precinct has some. Vast areas are 10+ min walk from food.</t>
+          <t>PARTIAL desert. 16 outlets for 30,000 workers (1:1,875). 3 are snack vans. Gatwick Rd strip has coverage, western half has nothing.</t>
         </is>
       </c>
       <c r="K3" s="33" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L3" s="32" t="n">
         <v>1</v>
       </c>
       <c r="M3" s="32" t="inlineStr">
         <is>
-          <t>UK's largest industrial BID. Organised management body to approach. £1.7bn GVA.</t>
+          <t>SCOUT VERIFIED. UK largest industrial BID. Gatwick Rd corridor has Subway, Starbucks, M&amp;S. But western/southern areas 15-20 min from food.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Slough Trading Estate</t>
         </is>
       </c>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Slough, Berkshire</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>SL1</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>M4 J6/J7, M25 J15</t>
         </is>
       </c>
-      <c r="E4" s="32" t="n">
+      <c r="E4" t="n">
         <v>353</v>
       </c>
-      <c r="F4" s="32" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>~13,000</t>
         </is>
       </c>
-      <c r="G4" s="32" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>~350</t>
         </is>
       </c>
-      <c r="H4" s="32" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Logistics, offices, light manufacturing, R&amp;D, data centres</t>
         </is>
       </c>
-      <c r="I4" s="32" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Mars, Dulux (AkzoNobel)</t>
         </is>
       </c>
-      <c r="J4" s="32" t="inlineStr">
-        <is>
-          <t>Some on-estate catering. Peripheral areas remote from shops.</t>
-        </is>
-      </c>
-      <c r="K4" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="L4" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" s="32" t="inlineStr">
-        <is>
-          <t>SEGRO-owned. 435 units. 24/7 warehouse operations.</t>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>NOT a food desert. 20 outlets inc Lidl, Iceland, 3 Greggs. Bordered by residential retail on Bath Rd + Farnham Rd.</t>
+        </is>
+      </c>
+      <c r="K4" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>SCOUT VERIFIED. Downgraded — adequate food coverage. Workers within 10 min walk of Greggs/Lidl/M&amp;S. Vending still viable in deep interior but less urgent.</t>
         </is>
       </c>
     </row>
@@ -12167,7 +12167,7 @@
       </c>
       <c r="J5" s="32" t="inlineStr">
         <is>
-          <t>Very poorly served. Enfield town centre 2 miles away.</t>
+          <t>PARTIAL desert. 7 outlets for 7,500 workers (1:1,071). Western half (Lockfield Ave, Brancroft Way) has zero food. 1 Greggs on Millmarsh Ln.</t>
         </is>
       </c>
       <c r="K5" s="33" t="n">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="M5" s="32" t="inlineStr">
         <is>
-          <t>London's 2nd largest industrial estate. £721m GVA. Multiple sub-estates.</t>
+          <t>SCOUT VERIFIED. London 2nd largest estate. Western interior is pure food desert. Green St edge has some options but long walk from interior.</t>
         </is>
       </c>
     </row>
@@ -12228,18 +12228,18 @@
       </c>
       <c r="J6" s="32" t="inlineStr">
         <is>
-          <t>Extremely isolated. Stanford-le-Hope 2 miles.</t>
+          <t>FOOD DESERT. 3 outlets on 1,500 acres. 1 warehouse cafe, 1 bistro, 1 Esso. Stanford-le-Hope 3 miles away. Car-dependent.</t>
         </is>
       </c>
       <c r="K6" s="33" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L6" s="32" t="n">
         <v>1</v>
       </c>
       <c r="M6" s="32" t="inlineStr">
         <is>
-          <t>24/7 port operations. 9M sq ft logistics park, 50% built. New 10-year expansion.</t>
+          <t>SCOUT VERIFIED. Extremely isolated. 24/7 port ops. No Greggs, no supermarket, no chains. Nearest proper shops 3 miles. Growing workforce.</t>
         </is>
       </c>
     </row>
@@ -12289,18 +12289,18 @@
       </c>
       <c r="J7" s="32" t="inlineStr">
         <is>
-          <t>Dartford town centre 3 miles. Limited on-site.</t>
+          <t>PARTIAL desert. 3 outlets in park (Costa + 2 restaurants). No grab-and-go beyond Costa. Stone village shops 10-15 min walk.</t>
         </is>
       </c>
       <c r="K7" s="33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L7" s="32" t="n">
         <v>1</v>
       </c>
       <c r="M7" s="32" t="inlineStr">
         <is>
-          <t>3M+ sq ft. Phase 2 adding 318,000 sq ft. 24/7 shift patterns.</t>
+          <t>SCOUT VERIFIED. Costa only quick food option. Restaurants serve sit-down meals not shift worker snacks. Stone village walkable but slow.</t>
         </is>
       </c>
     </row>
@@ -12408,7 +12408,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Some periphery retail. Estate itself is industrial.</t>
+          <t>PARTIAL desert on-site. 2 outlets (Greggs + Seven Seeded). Whippendell Rd shops ~10 min walk with Tesco Express, SPAR.</t>
         </is>
       </c>
       <c r="K9" s="21" t="n">
@@ -12419,7 +12419,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>New £25M development. Growing. Good mix of logistics and office.</t>
+          <t>SCOUT VERIFIED. Very thin on-site provision but smaller estate rescued by proximity to residential retail. On-site vending still valuable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 6 south London territories to planner (20 total)
Scouted south London industrial estates. Findings:
- Crayfields Park (BR5): confirmed food desert, but small (22 acres)
- Kimpton (SM3): food desert at 400m, unknown worker count
- Beddington Lane (CR0): partial desert in deep interior
- Willow Lane (CR4): NOT a desert — Tesco Express 254m
- Charlton Riverside (SE7): mixed, regeneration risk
- Purley Way (CR0): retail parks reduce isolation

South London lacks the mega-estates of the M25 corridor.
Best opportunities are single-machine placements, not clusters.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TheSnackChoice_London_Research.xlsx
+++ b/TheSnackChoice_London_Research.xlsx
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Product Catalog'!$A$1:$N$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Territory Planner'!$A$1:$M$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Territory Planner'!$A$1:$M$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -11853,7 +11853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12778,8 +12778,362 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>Willow Lane Trading Estate</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>Mitcham, CR4</t>
+        </is>
+      </c>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>CR4</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>A217/A237</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="n"/>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>2,500+</t>
+        </is>
+      </c>
+      <c r="G16" s="34" t="inlineStr">
+        <is>
+          <t>150+</t>
+        </is>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>Delivery, food manufacturing, electrical, glazing, demolition</t>
+        </is>
+      </c>
+      <c r="I16" s="34" t="inlineStr">
+        <is>
+          <t>Various SME (BID managed)</t>
+        </is>
+      </c>
+      <c r="J16" s="34" t="inlineStr">
+        <is>
+          <t>SCOUT: NOT a desert. 17 outlets within 800m. Tesco Express 254m. Mitcham town nearby.</t>
+        </is>
+      </c>
+      <c r="K16" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" s="34" t="inlineStr">
+        <is>
+          <t>SCOUT VERIFIED. Has own BID (willowlane.org.uk). Decent worker count but food access too good for vending to be essential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Beddington Lane Corridor</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Croydon, CR0</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CR0</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>M25 J7 (~6 miles)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1,000+ (est.)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Multiple sub-estates</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Logistics, distribution, warehousing</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>UPS, Morgan Stanley, Kuehne+Nagel, Asda, DPD, Amazon</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>SCOUT: PARTIAL desert. Deep Beddington Lane has 1 cafe at 400m, nothing else. Purley Way retail edge accessible but not walkable from interior.</t>
+        </is>
+      </c>
+      <c r="K17" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>SCOUT VERIFIED. Sub-estates: Prologis Park, SEGRO Park Croydon, Beddington TE, Silverwing. Major logistics = shift workers. Interior pockets isolated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Crayfields Park</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Orpington, BR5</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BR5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>M25 J4 (~5 miles)</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>22</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Several hundred (est.)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>14 units</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Mixed — offices, R&amp;D, industrial</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Stearn Electric, Euro Car Parts, London Ambulance Service</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>SCOUT: FOOD DESERT. 0 outlets within 800m. Nearest Londis 1km+. Nugent Retail Park 1km away.</t>
+        </is>
+      </c>
+      <c r="K18" s="21" t="n">
+        <v>7</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>SCOUT VERIFIED. Confirmed food desert but small scale (22 acres, 14 units). 1-2 machine opportunity, not a cluster play.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Kimpton Industrial Estate</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sutton, SM3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SM3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Via A217</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>30+ units across sub-estates</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Trade counters, warehousing, light industrial</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Various SME</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>SCOUT: FOOD DESERT at 400m. 2 outlets within 800m (both cafes 600m+). No convenience store or supermarket.</t>
+        </is>
+      </c>
+      <c r="K19" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>SCOUT VERIFIED. Food desert confirmed but worker count unknown. Sub-estates: iO Centre (20 units), Kimpton Trade &amp; Business Centre. Needs ground visit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>Charlton Riverside</t>
+        </is>
+      </c>
+      <c r="B20" s="34" t="inlineStr">
+        <is>
+          <t>Greenwich, SE7/SE18</t>
+        </is>
+      </c>
+      <c r="C20" s="34" t="inlineStr">
+        <is>
+          <t>SE7</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="inlineStr">
+        <is>
+          <t>Via A102/Blackwall Tunnel</t>
+        </is>
+      </c>
+      <c r="E20" s="34" t="n"/>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G20" s="34" t="inlineStr">
+        <is>
+          <t>~400</t>
+        </is>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>Industrial, distribution, aggregates</t>
+        </is>
+      </c>
+      <c r="I20" s="34" t="inlineStr">
+        <is>
+          <t>Aggregate Industries, Sainsburys distribution</t>
+        </is>
+      </c>
+      <c r="J20" s="34" t="inlineStr">
+        <is>
+          <t>Mixed — IKEA and Sainsburys now present but pockets remain industrial.</t>
+        </is>
+      </c>
+      <c r="K20" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" s="34" t="inlineStr">
+        <is>
+          <t>Not scouted. 400 businesses but regeneration risk — Westminster Industrial Estate converting to 450 homes. Target remaining pure-industrial pockets only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="34" t="inlineStr">
+        <is>
+          <t>Purley Way Corridor</t>
+        </is>
+      </c>
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>Croydon/Waddon, CR0</t>
+        </is>
+      </c>
+      <c r="C21" s="34" t="inlineStr">
+        <is>
+          <t>CR0</t>
+        </is>
+      </c>
+      <c r="D21" s="34" t="inlineStr">
+        <is>
+          <t>M25 J7 (~6 miles)</t>
+        </is>
+      </c>
+      <c r="E21" s="34" t="n"/>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G21" s="34" t="inlineStr">
+        <is>
+          <t>50+ across sub-estates</t>
+        </is>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>Industrial, retail parks, warehousing, logistics</t>
+        </is>
+      </c>
+      <c r="I21" s="34" t="inlineStr">
+        <is>
+          <t>Amazon, DPD, DHL, Royal Mail, Bookers</t>
+        </is>
+      </c>
+      <c r="J21" s="34" t="inlineStr">
+        <is>
+          <t>MODERATE — retail parks (IKEA, Costco) along the corridor provide food access. Industrial pockets may be isolated.</t>
+        </is>
+      </c>
+      <c r="K21" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="L21" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="M21" s="34" t="inlineStr">
+        <is>
+          <t>Not density-scouted separately. Adjacent retail parks reduce food isolation. Target specific industrial sub-estates (Valley IP, Beddington TE) not the whole corridor.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M20"/>
+  <autoFilter ref="A1:M21"/>
   <dataValidations count="1">
     <dataValidation sqref="L2:L50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Entry" error="Please select from the dropdown list" type="list">
       <formula1>"1,2,3"</formula1>

</xml_diff>

<commit_message>
feat: pre-populate Location Tracker with 16 Croydon-area leads
Romell is Croydon-based — reprioritised territories for SE London.
Location Tracker now has 16 pre-qualified leads along one restock route:

- 3 industrial sites (Beddington Lane corridor, Kimpton)
- 4 gyms (Kings Gym, WIZFIT, Gym Beast, Snap Fitness)
- 3 leisure venues (Oxygen, Kidspace, CroyWall, Airjump)
- 3 car dealerships (Mercedes, BMW, Toyota on Purley Way)

All within 3-8 miles of Croydon. Mix of spatial captivity (industrial)
and temporal captivity (gyms, leisure, dealership waiting areas).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TheSnackChoice_London_Research.xlsx
+++ b/TheSnackChoice_London_Research.xlsx
@@ -966,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1102,6 +1102,902 @@
       <c r="V1" s="15" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Beddington Lane — Prologis Park units</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Beddington Lane</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CR0 4TD</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Industrial/Warehouse</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>200</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T2" s="10" t="n">
+        <v>250</v>
+      </c>
+      <c r="U2" t="n">
+        <v>8</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>SEGRO/Prologis logistics units. UPS, Morgan Stanley. Shift workers, partial food desert confirmed by scout. Start here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Beddington Lane — Silverwing Industrial Estate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Horatius Way</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CR0 4RU</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Industrial/Warehouse</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>100</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T3" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="U3" t="n">
+        <v>7</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Gated secure estate. Multiple industrial units. Workers unlikely to walk to Purley Way during breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Beddington Trading Estate</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bath House Road</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CR0 4TT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Industrial/Warehouse</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>150</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T4" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="U4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Capital Industrial landlord. 15 units. 0.5mi from Purley Way retail but industrial roads = not walkable during breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Oxygen Trampoline Park</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>The Colonnades, 619 Purley Way</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CR0 4RQ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Leisure Centre</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>400</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Revenue share 10-15%</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="U5" t="n">
+        <v>9</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2,125 reviews. Families captive 1-2hrs. Kids = impulse buying. Temporal captivity. Check existing vending before approach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Kidspace Croydon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>The Colonnades, 619 Purley Way</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CR0 4RQ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Leisure Centre</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>300</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Revenue share 10-15%</t>
+        </is>
+      </c>
+      <c r="T6" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="U6" t="n">
+        <v>8</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>1,706 reviews. Soft play. Same retail park as Oxygen. Approach both together — one visit, two pitches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CroyWall Climbing Centre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Unit 7, New South Quarter, Whitestone Way</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CR0 4WN</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Leisure Centre</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>150</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T7" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="U7" t="n">
+        <v>7</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>454 reviews. Climbing = thirsty + hungry after. Industrial unit on Purley Way corridor. Water + protein bars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kings Gym Croydon</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Purley Way</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CR0 4RG</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>150</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T8" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="U8" t="n">
+        <v>7</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Small chain (Kings Gyms). Purley Way location. Protein bars + water + energy drinks. Romell's Snack Choice already does gyms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WIZFIT Studios</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>520a Purley Way</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CR0 4RE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>80</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T9" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="U9" t="n">
+        <v>6</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Independent. 140 reviews. Smaller gym but on the Purley Way restock route — marginal cost to service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gym Beast</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>93 Lower Addiscombe Rd</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CR0 6PT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>100</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T10" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="U10" t="n">
+        <v>7</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Independent. 319 reviews, 5.0 rating. High engagement = loyal members. Protein + water play.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz Croydon</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>76-78 Purley Way</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CR0 3JP</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>50</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="U11" t="n">
+        <v>6</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Car dealership service centre. Customers wait 1-4hrs. Micro-market in waiting area. On the Purley Way route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Berry Croydon BMW</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>57 Croydon Rd, Beddington</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CR0 4QE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>50</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T12" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="U12" t="n">
+        <v>6</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>BMW service centre. Beddington Lane area — same route as industrial sites. Temporal captivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Jemca Toyota Service Centre</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>57 Imperial Way</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CR0 4RR</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>40</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T13" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="U13" t="n">
+        <v>5</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Dedicated service site (separate from showroom). Imperial Way industrial area. Same route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Snap Fitness Wallington</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>93B Manor Rd</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SM6 0AT</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sutton</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>100</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T14" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="U14" t="n">
+        <v>6</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Small chain (Snap). 2mi from Beddington. On route to Kimpton/Sutton.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Airjump Trampoline Park</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>5A Lagoon Rd</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BR5 3QX</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Bromley</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Leisure Centre</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>200</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Revenue share 10-15%</t>
+        </is>
+      </c>
+      <c r="T15" s="10" t="n">
+        <v>250</v>
+      </c>
+      <c r="U15" t="n">
+        <v>8</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Independent. 625 reviews. ON Lagoon Rd industrial estate — adjacent to Crayfields. Families captive 1-2hrs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Fordes Gym</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>175 High St, St Mary Cray</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BR5 4AX</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Bromley</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>80</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T16" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="U16" t="n">
+        <v>6</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Independent. 2mi from Crayfields. Orpington cluster play if expanding east.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Kimpton Industrial Estate — iO Centre</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Minden Road</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SM3 9BL</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sutton</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Industrial/Warehouse</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>100</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Free placement</t>
+        </is>
+      </c>
+      <c r="T17" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="U17" t="n">
+        <v>7</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Scout confirmed food desert at 400m. 20 units. Trade counters + warehousing. 5mi from Croydon.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Croydon pivot — update strategy, report, and notes
Romell is Croydon-based. All deliverables updated:

Strategy Notes — 3 new sections:
- Croydon Base territory prioritisation (proximity > market size)
- Temporal captivity thesis (gyms, dealerships, leisure = time-stuck)
- The Croydon Corridor target route (16 leads mapped)

HTML Report — callouts and strategy updated for Croydon corridor,
dual captivity model (spatial + temporal), and mixed location types.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TheSnackChoice_London_Research.xlsx
+++ b/TheSnackChoice_London_Research.xlsx
@@ -3861,7 +3861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A108"/>
+  <dimension ref="A1:A154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -4367,61 +4367,306 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>THE BEHOLD LOOP (HOW TO IMPROVE)</t>
+          <t>CROYDON BASE — TERRITORY PRIORITISATION</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Monthly review cycle — built into the Performance Review sheet:</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  OBSERVE — What does the data say? (sales, margins, vend counts)</t>
+          <t>Romell is Croydon-based. The operator doing weekly restocks lives SE London.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>This changes the territory ranking completely — route efficiency depends on proximity to base.</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ORIENT — What does this mean? (bad location or bad product mix?)</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  DECIDE — What will you change? (one thing at a time)</t>
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>DECISION: Prioritise the Croydon corridor over Park Royal (NW10) and Brimsdown (EN3).</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ACT — Do it. Log it in the Operations Log.</t>
+          <t xml:space="preserve">  Beddington Lane:        2 miles from Croydon — home turf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="14" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Purley Way leisure:      3 miles — same corridor</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Kimpton, Sutton:         5 miles — quick run south</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Crayfields, Orpington:   8 miles — expansion east</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Park Royal:             12 miles, wrong side of London — deprioritised</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Manor Royal, Crawley:   25 miles south — day trip, not daily route</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Park Royal is the best market but Beddington is the best business decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Revenue per operator-HOUR matters more than revenue per machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>TEMPORAL CAPTIVITY — BEYOND INDUSTRIAL ESTATES</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Industrial estates are 'spatial captivity' — workers can't walk to food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>But there's a second type: 'temporal captivity' — people stuck for a time window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gyms:             Post-workout, sweaty, want protein NOW. 1-2hr window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Car dealerships:   Waiting 1-4hrs for service. Bored, nothing to do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Trampoline parks:  Kids on trampolines for 2hrs. Parents buy snacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Soft play:         Same as above. Impulse buying from captive parents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Climbing walls:    Thirsty + hungry after. Water + protein bars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>These aren't food deserts — there are shops nearby. But people can't or won't leave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>The Purley Way corridor combines both: Beddington Lane (spatial) + Oxygen/Kidspace (temporal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="13" t="inlineStr">
+        <is>
+          <t>DECISION: Mix location types along the same restock route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>One trip serves industrial units AND gyms AND leisure venues AND dealerships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>THE CROYDON CORRIDOR — TARGET ROUTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>16 pre-qualified leads in the Location Tracker, all on one route:</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. Beddington Lane industrial (3 sites) — spatial captivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. Purley Way dealerships (3 sites) — temporal captivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. Purley Way leisure (Oxygen, Kidspace, CroyWall) — temporal captivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. Kings Gym / WIZFIT (2 gyms on route) — temporal captivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5. Gym Beast, Snap Fitness (2 more gyms nearby) — temporal captivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  6. Kimpton Industrial Estate (1 site, Sutton) — spatial captivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7. Airjump + Fordes Gym (Orpington, expansion) — temporal captivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>5-7 sites achievable in phase 1. All within 30 minutes driving of Croydon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Est. weekly revenue: £1,200-1,800 across the cluster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>THE BEHOLD LOOP (HOW TO IMPROVE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Monthly review cycle — built into the Performance Review sheet:</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OBSERVE — What does the data say? (sales, margins, vend counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ORIENT — What does this mean? (bad location or bad product mix?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DECIDE — What will you change? (one thing at a time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ACT — Do it. Log it in the Operations Log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="14" t="inlineStr">
+        <is>
           <t xml:space="preserve">  PROTECT — What could go wrong? (stock-out risk, customer complaints?)</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="13" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="13" t="inlineStr">
         <is>
           <t>KEY RULE: One change at a time. Wait 4 weeks. Then measure.</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
+    <row r="154">
+      <c r="A154" t="inlineStr">
         <is>
           <t>If you change two things at once, you can't tell which one worked.</t>
         </is>

</xml_diff>